<commit_message>
Accept mission AW-20260908-002 homepage concept revision
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R759f463e05174d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R7c80c03efec24de0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R4fb68172a19b40cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Redbacb37fcfd44ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Rb34a894e2db3414e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Rcbeade6ffe3242f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,6 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
@@ -97,7 +100,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -125,6 +128,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1214,6 +1223,23 @@
         <x:v>ACCEPTED — root-path deployment artifact ready for authorized publication</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="112.5" hidden="0" customHeight="1">
+      <x:c r="A29" s="11" t="n">
+        <x:v>46273.5</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>Mission AW-20260908-002 — Homepage Sections 05–06 conceptual revision</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>Accepted actor commit 5db4b630896bfb0a4e5289fb72b5ea9164b4cad1. Exact approved copy and six landscape elements are present; Technology and Intelligence were removed from the landscape; Section 06 explains the understanding before introducing CIE. Root and repository-subpath suites each passed 31/31.</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
+        <x:v>0 new defects</x:v>
+      </x:c>
+      <x:c r="E29" s="10" t="str">
+        <x:v>ACCEPTED — bounded Sections 05–06 revision; not pushed or deployed</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2579,7 +2605,32 @@
         <x:v>Accepted by Codex disposition of AW-20260904-005 at b51db15. Actor scope was limited to the workflow and its return artifact; DNS, repository settings, push, and live publication remain separate authorized operator actions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="18" customHeight="1"/>
+    <x:row r="36" ht="138.75" hidden="0" customHeight="1">
+      <x:c r="A36" s="11" t="n">
+        <x:v>46273.5</x:v>
+      </x:c>
+      <x:c r="B36" s="10" t="str">
+        <x:v>Homepage / Capability landscape and CIE definition</x:v>
+      </x:c>
+      <x:c r="C36" s="10" t="str">
+        <x:v>src/pages/home.mjs + src/assets/home.css + src/assets/alaya-05-living-field-*.svg</x:v>
+      </x:c>
+      <x:c r="D36" s="10" t="str">
+        <x:v>Sections 05–06 now present capability as living terrain with Experience, Practice, Contribution, Knowledge and Curiosity in one field, then define Capability Intelligence before introducing CIE.</x:v>
+      </x:c>
+      <x:c r="E36" s="10" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F36" s="10" t="str">
+        <x:v>Retain the six-element landscape, exact approved definition order, responsive containment, decorative artwork treatment and unchanged Section 06 maturity content.</x:v>
+      </x:c>
+      <x:c r="G36" s="10" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="H36" s="10" t="str">
+        <x:v>Accepted by Codex disposition for AW-20260908-002 at actor commit 5db4b630896bfb0a4e5289fb72b5ea9164b4cad1. Root and /alaya-crafts-website suites passed 31/31. No push or deployment.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="37" ht="18" customHeight="1"/>
     <x:row r="38" ht="18" customHeight="1"/>
     <x:row r="39" ht="18" customHeight="1"/>

</xml_diff>